<commit_message>
Updated Excel code format
</commit_message>
<xml_diff>
--- a/Codes/benchmark_winrates.xlsx
+++ b/Codes/benchmark_winrates.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rgdar\OneDrive\Desktop\Academics\ASC\Final-Year-Project\Codes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C2D488B-63DB-4956-9ED7-E53F9D4E3D5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6696575F-4C74-4BD6-B5F6-C4FFA296CB42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Win Rates" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>Algorithm</t>
   </si>
@@ -28,6 +28,12 @@
     <t>Run1</t>
   </si>
   <si>
+    <t>Run2</t>
+  </si>
+  <si>
+    <t>Run3</t>
+  </si>
+  <si>
     <t>CCE-TDCCEA</t>
   </si>
   <si>
@@ -58,7 +64,13 @@
     <t>SA-PDCoEA</t>
   </si>
   <si>
-    <t>Run2</t>
+    <t>Time1</t>
+  </si>
+  <si>
+    <t>Time2</t>
+  </si>
+  <si>
+    <t>Time3</t>
   </si>
 </sst>
 </file>
@@ -398,14 +410,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.109375" customWidth="1"/>
-    <col min="2" max="2" width="12.33203125" customWidth="1"/>
+    <col min="2" max="3" width="12.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -413,117 +425,249 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+        <v>14</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B2">
         <v>71.430000000000007</v>
       </c>
       <c r="C2">
+        <v>815.5</v>
+      </c>
+      <c r="D2">
         <v>91.4</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>85.71</v>
+      </c>
+      <c r="G2">
+        <v>915.3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B3">
         <v>100</v>
       </c>
       <c r="C3">
+        <v>869.7</v>
+      </c>
+      <c r="D3">
         <v>85.7</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>62.86</v>
+      </c>
+      <c r="G3">
+        <v>978</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B4">
         <v>68.569999999999993</v>
       </c>
       <c r="C4">
+        <v>250.7</v>
+      </c>
+      <c r="D4">
         <v>62.9</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>14.29</v>
+      </c>
+      <c r="G4">
+        <v>135.80000000000001</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B5">
         <v>80</v>
       </c>
       <c r="C5">
+        <v>137.80000000000001</v>
+      </c>
+      <c r="D5">
         <v>42.9</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>68.569999999999993</v>
+      </c>
+      <c r="G5">
+        <v>159.1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B6">
         <v>57.14</v>
       </c>
       <c r="C6">
+        <v>167.8</v>
+      </c>
+      <c r="D6">
         <v>31.4</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <v>80</v>
+      </c>
+      <c r="G6">
+        <v>165.9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B7">
         <v>14.29</v>
       </c>
       <c r="C7">
+        <v>159.30000000000001</v>
+      </c>
+      <c r="D7">
         <v>14.3</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <v>51.43</v>
+      </c>
+      <c r="G7">
+        <v>182.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B8">
         <v>57.14</v>
       </c>
       <c r="C8">
+        <v>119.1</v>
+      </c>
+      <c r="D8">
         <v>71.400000000000006</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>45.71</v>
+      </c>
+      <c r="G8">
+        <v>174.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B9">
         <v>85.71</v>
       </c>
       <c r="C9">
+        <v>145.80000000000001</v>
+      </c>
+      <c r="D9">
         <v>85.7</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <v>28.57</v>
+      </c>
+      <c r="G9">
+        <v>163.19999999999999</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B10">
         <v>57.14</v>
       </c>
       <c r="C10">
+        <v>115.5</v>
+      </c>
+      <c r="D10">
         <v>51.4</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>57.14</v>
+      </c>
+      <c r="G10">
+        <v>137.80000000000001</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B11">
         <v>85.71</v>
       </c>
       <c r="C11">
+        <v>0</v>
+      </c>
+      <c r="D11">
         <v>71.400000000000006</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+      <c r="F11">
+        <v>71.430000000000007</v>
+      </c>
+      <c r="G11">
+        <v>1885.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>